<commit_message>
update additional criteria columns and bug fix
</commit_message>
<xml_diff>
--- a/inst/extdata/south_dakota_criteria_crosswalk.xlsx
+++ b/inst/extdata/south_dakota_criteria_crosswalk.xlsx
@@ -1,20 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://tetratechinc-my.sharepoint.com/personal/k_salkgundersen_tetratech_com/Documents/EPA/R8_AssessmentTool/5_Work/Crosswalks/individual_criteria_crosswalks/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kwong01\TADACommunityHub\inst\extdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6CC4534E-B8EE-4EAC-A9EE-2BFCB51221B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EADE0E40-1828-48B8-B02B-0ECB66DD172B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{5F38D7ED-F210-48EE-9D63-71C5059EEFD4}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{5F38D7ED-F210-48EE-9D63-71C5059EEFD4}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$AQ$272</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -33,6 +36,33 @@
     </ext>
   </extLst>
 </workbook>
+</file>
+
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>tc={D4650B53-0A04-4080-9477-D3AA35554A29}</author>
+    <author>tc={366934B1-F374-42FE-9238-A6CCE9E3FAB1}</author>
+  </authors>
+  <commentList>
+    <comment ref="Q15" authorId="0" shapeId="0" xr:uid="{D4650B53-0A04-4080-9477-D3AA35554A29}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    30</t>
+      </text>
+    </comment>
+    <comment ref="U15" authorId="1" shapeId="0" xr:uid="{366934B1-F374-42FE-9238-A6CCE9E3FAB1}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    If the magnitude value cannot be exceeded at all during this 30 day period</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
@@ -690,7 +720,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -727,13 +757,25 @@
       <family val="2"/>
       <charset val="136"/>
     </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -748,7 +790,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -763,6 +805,9 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -780,6 +825,12 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <person displayName="Wong, Kenny" id="{3B9F0CFB-71E0-49B7-A614-E93A7328F0E9}" userId="S::Wong.Kenny@epa.gov::22d39ba2-7a17-454f-a1e0-b7fc51176133" providerId="AD"/>
+</personList>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1097,12 +1148,28 @@
 </a:theme>
 </file>
 
+<file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
+<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="Q15" dT="2025-12-22T18:09:06.05" personId="{3B9F0CFB-71E0-49B7-A614-E93A7328F0E9}" id="{D4650B53-0A04-4080-9477-D3AA35554A29}">
+    <text>30</text>
+  </threadedComment>
+  <threadedComment ref="U15" dT="2025-12-22T18:09:38.04" personId="{3B9F0CFB-71E0-49B7-A614-E93A7328F0E9}" id="{366934B1-F374-42FE-9238-A6CCE9E3FAB1}">
+    <text>If the magnitude value cannot be exceeded at all during this 30 day period</text>
+  </threadedComment>
+</ThreadedComments>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C3395A04-AF43-4335-9FBC-13D8E09A4DF0}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C3395A04-AF43-4335-9FBC-13D8E09A4DF0}">
   <dimension ref="A1:AQ272"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="19" max="19" width="18.90625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="27.7265625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="15.26953125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:43" s="4" customFormat="1" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:43" s="4" customFormat="1" ht="46.5" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1233,7 +1300,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="2" spans="1:43" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:43" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A2" s="5"/>
       <c r="B2" s="5" t="s">
         <v>43</v>
@@ -1302,7 +1369,7 @@
       <c r="AL2" s="5"/>
       <c r="AM2" s="5"/>
     </row>
-    <row r="3" spans="1:43" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:43" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A3" s="5"/>
       <c r="B3" s="5" t="s">
         <v>43</v>
@@ -1371,7 +1438,7 @@
       <c r="AL3" s="5"/>
       <c r="AM3" s="5"/>
     </row>
-    <row r="4" spans="1:43" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:43" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A4" s="5"/>
       <c r="B4" s="5" t="s">
         <v>43</v>
@@ -1438,7 +1505,7 @@
       <c r="AL4" s="5"/>
       <c r="AM4" s="5"/>
     </row>
-    <row r="5" spans="1:43" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:43" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A5" s="5"/>
       <c r="B5" s="5" t="s">
         <v>43</v>
@@ -1505,7 +1572,7 @@
       <c r="AL5" s="5"/>
       <c r="AM5" s="5"/>
     </row>
-    <row r="6" spans="1:43" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:43" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A6" s="5"/>
       <c r="B6" s="5" t="s">
         <v>43</v>
@@ -1572,7 +1639,7 @@
       <c r="AL6" s="5"/>
       <c r="AM6" s="5"/>
     </row>
-    <row r="7" spans="1:43" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:43" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A7" s="5"/>
       <c r="B7" s="5" t="s">
         <v>43</v>
@@ -1639,7 +1706,7 @@
       <c r="AL7" s="5"/>
       <c r="AM7" s="5"/>
     </row>
-    <row r="8" spans="1:43" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:43" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A8" s="5"/>
       <c r="B8" s="5" t="s">
         <v>43</v>
@@ -1706,7 +1773,7 @@
       <c r="AL8" s="5"/>
       <c r="AM8" s="5"/>
     </row>
-    <row r="9" spans="1:43" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:43" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A9" s="5"/>
       <c r="B9" s="5" t="s">
         <v>43</v>
@@ -1773,7 +1840,7 @@
       <c r="AL9" s="5"/>
       <c r="AM9" s="5"/>
     </row>
-    <row r="10" spans="1:43" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:43" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A10" s="5"/>
       <c r="B10" s="5" t="s">
         <v>43</v>
@@ -1840,7 +1907,7 @@
       <c r="AL10" s="5"/>
       <c r="AM10" s="5"/>
     </row>
-    <row r="11" spans="1:43" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:43" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A11" s="5"/>
       <c r="B11" s="5" t="s">
         <v>43</v>
@@ -1911,7 +1978,7 @@
       <c r="AL11" s="5"/>
       <c r="AM11" s="5"/>
     </row>
-    <row r="12" spans="1:43" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:43" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A12" s="5"/>
       <c r="B12" s="5" t="s">
         <v>43</v>
@@ -1982,7 +2049,7 @@
       <c r="AL12" s="5"/>
       <c r="AM12" s="5"/>
     </row>
-    <row r="13" spans="1:43" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:43" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A13" s="5"/>
       <c r="B13" s="5" t="s">
         <v>43</v>
@@ -2053,7 +2120,7 @@
       <c r="AL13" s="5"/>
       <c r="AM13" s="5"/>
     </row>
-    <row r="14" spans="1:43" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:43" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A14" s="5"/>
       <c r="B14" s="5" t="s">
         <v>43</v>
@@ -2124,7 +2191,7 @@
       <c r="AL14" s="5"/>
       <c r="AM14" s="5"/>
     </row>
-    <row r="15" spans="1:43" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:43" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A15" s="5"/>
       <c r="B15" s="5" t="s">
         <v>43</v>
@@ -2169,7 +2236,7 @@
       <c r="T15" s="5">
         <v>1</v>
       </c>
-      <c r="U15" s="5" t="s">
+      <c r="U15" s="6" t="s">
         <v>74</v>
       </c>
       <c r="V15" s="5"/>
@@ -2195,7 +2262,7 @@
       <c r="AL15" s="5"/>
       <c r="AM15" s="5"/>
     </row>
-    <row r="16" spans="1:43" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:43" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A16" s="5"/>
       <c r="B16" s="5" t="s">
         <v>43</v>
@@ -2240,7 +2307,7 @@
       <c r="T16" s="5">
         <v>1</v>
       </c>
-      <c r="U16" s="5" t="s">
+      <c r="U16" s="6" t="s">
         <v>74</v>
       </c>
       <c r="V16" s="5"/>
@@ -2266,7 +2333,7 @@
       <c r="AL16" s="5"/>
       <c r="AM16" s="5"/>
     </row>
-    <row r="17" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A17" s="5"/>
       <c r="B17" s="5" t="s">
         <v>43</v>
@@ -2311,7 +2378,7 @@
       <c r="T17" s="5">
         <v>1</v>
       </c>
-      <c r="U17" s="5" t="s">
+      <c r="U17" s="6" t="s">
         <v>74</v>
       </c>
       <c r="V17" s="5"/>
@@ -2337,7 +2404,7 @@
       <c r="AL17" s="5"/>
       <c r="AM17" s="5"/>
     </row>
-    <row r="18" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A18" s="5"/>
       <c r="B18" s="5" t="s">
         <v>43</v>
@@ -2382,7 +2449,7 @@
       <c r="T18" s="5">
         <v>1</v>
       </c>
-      <c r="U18" s="5" t="s">
+      <c r="U18" s="6" t="s">
         <v>74</v>
       </c>
       <c r="V18" s="5"/>
@@ -2408,7 +2475,7 @@
       <c r="AL18" s="5"/>
       <c r="AM18" s="5"/>
     </row>
-    <row r="19" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A19" s="5"/>
       <c r="B19" s="5" t="s">
         <v>43</v>
@@ -2477,7 +2544,7 @@
       <c r="AL19" s="5"/>
       <c r="AM19" s="5"/>
     </row>
-    <row r="20" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A20" s="5"/>
       <c r="B20" s="5" t="s">
         <v>43</v>
@@ -2546,7 +2613,7 @@
       <c r="AL20" s="5"/>
       <c r="AM20" s="5"/>
     </row>
-    <row r="21" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A21" s="5"/>
       <c r="B21" s="5" t="s">
         <v>43</v>
@@ -2615,7 +2682,7 @@
       <c r="AL21" s="5"/>
       <c r="AM21" s="5"/>
     </row>
-    <row r="22" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A22" s="5"/>
       <c r="B22" s="5" t="s">
         <v>43</v>
@@ -2684,7 +2751,7 @@
       <c r="AL22" s="5"/>
       <c r="AM22" s="5"/>
     </row>
-    <row r="23" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A23" s="5"/>
       <c r="B23" s="5" t="s">
         <v>43</v>
@@ -2751,7 +2818,7 @@
       <c r="AL23" s="5"/>
       <c r="AM23" s="5"/>
     </row>
-    <row r="24" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A24" s="5"/>
       <c r="B24" s="5" t="s">
         <v>43</v>
@@ -2820,7 +2887,7 @@
       <c r="AL24" s="5"/>
       <c r="AM24" s="5"/>
     </row>
-    <row r="25" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A25" s="5"/>
       <c r="B25" s="5" t="s">
         <v>43</v>
@@ -2889,7 +2956,7 @@
       <c r="AL25" s="5"/>
       <c r="AM25" s="5"/>
     </row>
-    <row r="26" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A26" s="5"/>
       <c r="B26" s="5" t="s">
         <v>43</v>
@@ -2958,7 +3025,7 @@
       <c r="AL26" s="5"/>
       <c r="AM26" s="5"/>
     </row>
-    <row r="27" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A27" s="5"/>
       <c r="B27" s="5" t="s">
         <v>43</v>
@@ -3027,7 +3094,7 @@
       <c r="AL27" s="5"/>
       <c r="AM27" s="5"/>
     </row>
-    <row r="28" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A28" s="5"/>
       <c r="B28" s="5" t="s">
         <v>43</v>
@@ -3096,7 +3163,7 @@
       <c r="AL28" s="5"/>
       <c r="AM28" s="5"/>
     </row>
-    <row r="29" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A29" s="5"/>
       <c r="B29" s="5" t="s">
         <v>43</v>
@@ -3163,7 +3230,7 @@
       <c r="AL29" s="5"/>
       <c r="AM29" s="5"/>
     </row>
-    <row r="30" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A30" s="5"/>
       <c r="B30" s="5" t="s">
         <v>43</v>
@@ -3230,7 +3297,7 @@
       <c r="AL30" s="5"/>
       <c r="AM30" s="5"/>
     </row>
-    <row r="31" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A31" s="5"/>
       <c r="B31" s="5" t="s">
         <v>43</v>
@@ -3297,7 +3364,7 @@
       <c r="AL31" s="5"/>
       <c r="AM31" s="5"/>
     </row>
-    <row r="32" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A32" s="5"/>
       <c r="B32" s="5" t="s">
         <v>43</v>
@@ -3368,7 +3435,7 @@
       <c r="AL32" s="5"/>
       <c r="AM32" s="5"/>
     </row>
-    <row r="33" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A33" s="5"/>
       <c r="B33" s="5" t="s">
         <v>43</v>
@@ -3439,7 +3506,7 @@
       <c r="AL33" s="5"/>
       <c r="AM33" s="5"/>
     </row>
-    <row r="34" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A34" s="5"/>
       <c r="B34" s="5" t="s">
         <v>43</v>
@@ -3510,7 +3577,7 @@
       <c r="AL34" s="5"/>
       <c r="AM34" s="5"/>
     </row>
-    <row r="35" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A35" s="5"/>
       <c r="B35" s="5" t="s">
         <v>43</v>
@@ -3581,7 +3648,7 @@
       <c r="AL35" s="5"/>
       <c r="AM35" s="5"/>
     </row>
-    <row r="36" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A36" s="5"/>
       <c r="B36" s="5" t="s">
         <v>43</v>
@@ -3652,7 +3719,7 @@
       <c r="AL36" s="5"/>
       <c r="AM36" s="5"/>
     </row>
-    <row r="37" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A37" s="5"/>
       <c r="B37" s="5" t="s">
         <v>43</v>
@@ -3723,7 +3790,7 @@
       <c r="AL37" s="5"/>
       <c r="AM37" s="5"/>
     </row>
-    <row r="38" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A38" s="5"/>
       <c r="B38" s="5" t="s">
         <v>43</v>
@@ -3796,7 +3863,7 @@
       <c r="AL38" s="5"/>
       <c r="AM38" s="5"/>
     </row>
-    <row r="39" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A39" s="5"/>
       <c r="B39" s="5" t="s">
         <v>43</v>
@@ -3869,7 +3936,7 @@
       <c r="AL39" s="5"/>
       <c r="AM39" s="5"/>
     </row>
-    <row r="40" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A40" s="5"/>
       <c r="B40" s="5" t="s">
         <v>43</v>
@@ -3940,7 +4007,7 @@
       <c r="AL40" s="5"/>
       <c r="AM40" s="5"/>
     </row>
-    <row r="41" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A41" s="5"/>
       <c r="B41" s="5" t="s">
         <v>43</v>
@@ -4011,7 +4078,7 @@
       <c r="AL41" s="5"/>
       <c r="AM41" s="5"/>
     </row>
-    <row r="42" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A42" s="5"/>
       <c r="B42" s="5" t="s">
         <v>43</v>
@@ -4080,7 +4147,7 @@
       <c r="AL42" s="5"/>
       <c r="AM42" s="5"/>
     </row>
-    <row r="43" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A43" s="5"/>
       <c r="B43" s="5" t="s">
         <v>43</v>
@@ -4149,7 +4216,7 @@
       <c r="AL43" s="5"/>
       <c r="AM43" s="5"/>
     </row>
-    <row r="44" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A44" s="5"/>
       <c r="B44" s="5" t="s">
         <v>43</v>
@@ -4218,7 +4285,7 @@
       <c r="AL44" s="5"/>
       <c r="AM44" s="5"/>
     </row>
-    <row r="45" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A45" s="5"/>
       <c r="B45" s="5" t="s">
         <v>43</v>
@@ -4287,7 +4354,7 @@
       <c r="AL45" s="5"/>
       <c r="AM45" s="5"/>
     </row>
-    <row r="46" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A46" s="5"/>
       <c r="B46" s="5" t="s">
         <v>43</v>
@@ -4356,7 +4423,7 @@
       <c r="AL46" s="5"/>
       <c r="AM46" s="5"/>
     </row>
-    <row r="47" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A47" s="5"/>
       <c r="B47" s="5" t="s">
         <v>43</v>
@@ -4425,7 +4492,7 @@
       <c r="AL47" s="5"/>
       <c r="AM47" s="5"/>
     </row>
-    <row r="48" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A48" s="5"/>
       <c r="B48" s="5" t="s">
         <v>43</v>
@@ -4494,7 +4561,7 @@
       <c r="AL48" s="5"/>
       <c r="AM48" s="5"/>
     </row>
-    <row r="49" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A49" s="5"/>
       <c r="B49" s="5" t="s">
         <v>43</v>
@@ -4563,7 +4630,7 @@
       <c r="AL49" s="5"/>
       <c r="AM49" s="5"/>
     </row>
-    <row r="50" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A50" s="5"/>
       <c r="B50" s="5" t="s">
         <v>43</v>
@@ -4630,7 +4697,7 @@
       <c r="AL50" s="5"/>
       <c r="AM50" s="5"/>
     </row>
-    <row r="51" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A51" s="5"/>
       <c r="B51" s="5" t="s">
         <v>43</v>
@@ -4701,7 +4768,7 @@
       <c r="AL51" s="5"/>
       <c r="AM51" s="5"/>
     </row>
-    <row r="52" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A52" s="5"/>
       <c r="B52" s="5" t="s">
         <v>43</v>
@@ -4770,7 +4837,7 @@
       <c r="AL52" s="5"/>
       <c r="AM52" s="5"/>
     </row>
-    <row r="53" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A53" s="5"/>
       <c r="B53" s="5" t="s">
         <v>43</v>
@@ -4839,7 +4906,7 @@
       <c r="AL53" s="5"/>
       <c r="AM53" s="5"/>
     </row>
-    <row r="54" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A54" s="5"/>
       <c r="B54" s="5" t="s">
         <v>43</v>
@@ -4908,7 +4975,7 @@
       <c r="AL54" s="5"/>
       <c r="AM54" s="5"/>
     </row>
-    <row r="55" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A55" s="5"/>
       <c r="B55" s="5" t="s">
         <v>43</v>
@@ -4977,7 +5044,7 @@
       <c r="AL55" s="5"/>
       <c r="AM55" s="5"/>
     </row>
-    <row r="56" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A56" s="5"/>
       <c r="B56" s="5" t="s">
         <v>43</v>
@@ -5046,7 +5113,7 @@
       <c r="AL56" s="5"/>
       <c r="AM56" s="5"/>
     </row>
-    <row r="57" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A57" s="5"/>
       <c r="B57" s="5" t="s">
         <v>43</v>
@@ -5115,7 +5182,7 @@
       <c r="AL57" s="5"/>
       <c r="AM57" s="5"/>
     </row>
-    <row r="58" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A58" s="5"/>
       <c r="B58" s="5" t="s">
         <v>43</v>
@@ -5184,7 +5251,7 @@
       <c r="AL58" s="5"/>
       <c r="AM58" s="5"/>
     </row>
-    <row r="59" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A59" s="5"/>
       <c r="B59" s="5" t="s">
         <v>43</v>
@@ -5253,7 +5320,7 @@
       <c r="AL59" s="5"/>
       <c r="AM59" s="5"/>
     </row>
-    <row r="60" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A60" s="5"/>
       <c r="B60" s="5" t="s">
         <v>43</v>
@@ -5322,7 +5389,7 @@
       <c r="AL60" s="5"/>
       <c r="AM60" s="5"/>
     </row>
-    <row r="61" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A61" s="5"/>
       <c r="B61" s="5" t="s">
         <v>43</v>
@@ -5391,7 +5458,7 @@
       <c r="AL61" s="5"/>
       <c r="AM61" s="5"/>
     </row>
-    <row r="62" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A62" s="5"/>
       <c r="B62" s="5" t="s">
         <v>43</v>
@@ -5460,7 +5527,7 @@
       <c r="AL62" s="5"/>
       <c r="AM62" s="5"/>
     </row>
-    <row r="63" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A63" s="5"/>
       <c r="B63" s="5" t="s">
         <v>43</v>
@@ -5529,7 +5596,7 @@
       <c r="AL63" s="5"/>
       <c r="AM63" s="5"/>
     </row>
-    <row r="64" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A64" s="5"/>
       <c r="B64" s="5" t="s">
         <v>43</v>
@@ -5598,7 +5665,7 @@
       <c r="AL64" s="5"/>
       <c r="AM64" s="5"/>
     </row>
-    <row r="65" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A65" s="5"/>
       <c r="B65" s="5" t="s">
         <v>43</v>
@@ -5667,7 +5734,7 @@
       <c r="AL65" s="5"/>
       <c r="AM65" s="5"/>
     </row>
-    <row r="66" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A66" s="5"/>
       <c r="B66" s="5" t="s">
         <v>43</v>
@@ -5736,7 +5803,7 @@
       <c r="AL66" s="5"/>
       <c r="AM66" s="5"/>
     </row>
-    <row r="67" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A67" s="5"/>
       <c r="B67" s="5" t="s">
         <v>43</v>
@@ -5803,7 +5870,7 @@
       <c r="AL67" s="5"/>
       <c r="AM67" s="5"/>
     </row>
-    <row r="68" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A68" s="5"/>
       <c r="B68" s="5" t="s">
         <v>43</v>
@@ -5870,7 +5937,7 @@
       <c r="AL68" s="5"/>
       <c r="AM68" s="5"/>
     </row>
-    <row r="69" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A69" s="5"/>
       <c r="B69" s="5" t="s">
         <v>43</v>
@@ -5937,7 +6004,7 @@
       <c r="AL69" s="5"/>
       <c r="AM69" s="5"/>
     </row>
-    <row r="70" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A70" s="5"/>
       <c r="B70" s="5" t="s">
         <v>43</v>
@@ -6004,7 +6071,7 @@
       <c r="AL70" s="5"/>
       <c r="AM70" s="5"/>
     </row>
-    <row r="71" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A71" s="5"/>
       <c r="B71" s="5" t="s">
         <v>43</v>
@@ -6071,7 +6138,7 @@
       <c r="AL71" s="5"/>
       <c r="AM71" s="5"/>
     </row>
-    <row r="72" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A72" s="5"/>
       <c r="B72" s="5" t="s">
         <v>43</v>
@@ -6138,7 +6205,7 @@
       <c r="AL72" s="5"/>
       <c r="AM72" s="5"/>
     </row>
-    <row r="73" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A73" s="5"/>
       <c r="B73" s="5" t="s">
         <v>43</v>
@@ -6205,7 +6272,7 @@
       <c r="AL73" s="5"/>
       <c r="AM73" s="5"/>
     </row>
-    <row r="74" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A74" s="5"/>
       <c r="B74" s="5" t="s">
         <v>43</v>
@@ -6272,7 +6339,7 @@
       <c r="AL74" s="5"/>
       <c r="AM74" s="5"/>
     </row>
-    <row r="75" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A75" s="5"/>
       <c r="B75" s="5" t="s">
         <v>43</v>
@@ -6341,7 +6408,7 @@
       <c r="AL75" s="5"/>
       <c r="AM75" s="5"/>
     </row>
-    <row r="76" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A76" s="5"/>
       <c r="B76" s="5" t="s">
         <v>43</v>
@@ -6410,7 +6477,7 @@
       <c r="AL76" s="5"/>
       <c r="AM76" s="5"/>
     </row>
-    <row r="77" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A77" s="5"/>
       <c r="B77" s="5" t="s">
         <v>43</v>
@@ -6479,7 +6546,7 @@
       <c r="AL77" s="5"/>
       <c r="AM77" s="5"/>
     </row>
-    <row r="78" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A78" s="5"/>
       <c r="B78" s="5" t="s">
         <v>43</v>
@@ -6548,7 +6615,7 @@
       <c r="AL78" s="5"/>
       <c r="AM78" s="5"/>
     </row>
-    <row r="79" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A79" s="5"/>
       <c r="B79" s="5" t="s">
         <v>43</v>
@@ -6617,7 +6684,7 @@
       <c r="AL79" s="5"/>
       <c r="AM79" s="5"/>
     </row>
-    <row r="80" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A80" s="5"/>
       <c r="B80" s="5" t="s">
         <v>43</v>
@@ -6690,7 +6757,7 @@
       <c r="AL80" s="5"/>
       <c r="AM80" s="5"/>
     </row>
-    <row r="81" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A81" s="5"/>
       <c r="B81" s="5" t="s">
         <v>43</v>
@@ -6763,7 +6830,7 @@
       <c r="AL81" s="5"/>
       <c r="AM81" s="5"/>
     </row>
-    <row r="82" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A82" s="5"/>
       <c r="B82" s="5" t="s">
         <v>43</v>
@@ -6836,7 +6903,7 @@
       <c r="AL82" s="5"/>
       <c r="AM82" s="5"/>
     </row>
-    <row r="83" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A83" s="5"/>
       <c r="B83" s="5" t="s">
         <v>43</v>
@@ -6909,7 +6976,7 @@
       <c r="AL83" s="5"/>
       <c r="AM83" s="5"/>
     </row>
-    <row r="84" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A84" s="5"/>
       <c r="B84" s="5" t="s">
         <v>43</v>
@@ -6982,7 +7049,7 @@
       <c r="AL84" s="5"/>
       <c r="AM84" s="5"/>
     </row>
-    <row r="85" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A85" s="5"/>
       <c r="B85" s="5" t="s">
         <v>43</v>
@@ -7055,7 +7122,7 @@
       <c r="AL85" s="5"/>
       <c r="AM85" s="5"/>
     </row>
-    <row r="86" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A86" s="5"/>
       <c r="B86" s="5" t="s">
         <v>43</v>
@@ -7128,7 +7195,7 @@
       <c r="AL86" s="5"/>
       <c r="AM86" s="5"/>
     </row>
-    <row r="87" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A87" s="5"/>
       <c r="B87" s="5" t="s">
         <v>43</v>
@@ -7201,7 +7268,7 @@
       <c r="AL87" s="5"/>
       <c r="AM87" s="5"/>
     </row>
-    <row r="88" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A88" s="5"/>
       <c r="B88" s="5" t="s">
         <v>43</v>
@@ -7274,7 +7341,7 @@
       <c r="AL88" s="5"/>
       <c r="AM88" s="5"/>
     </row>
-    <row r="89" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A89" s="5"/>
       <c r="B89" s="5" t="s">
         <v>43</v>
@@ -7347,7 +7414,7 @@
       <c r="AL89" s="5"/>
       <c r="AM89" s="5"/>
     </row>
-    <row r="90" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A90" s="5"/>
       <c r="B90" s="5" t="s">
         <v>43</v>
@@ -7414,7 +7481,7 @@
       <c r="AL90" s="5"/>
       <c r="AM90" s="5"/>
     </row>
-    <row r="91" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A91" s="5"/>
       <c r="B91" s="5" t="s">
         <v>43</v>
@@ -7481,7 +7548,7 @@
       <c r="AL91" s="5"/>
       <c r="AM91" s="5"/>
     </row>
-    <row r="92" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A92" s="5"/>
       <c r="B92" s="5" t="s">
         <v>43</v>
@@ -7548,7 +7615,7 @@
       <c r="AL92" s="5"/>
       <c r="AM92" s="5"/>
     </row>
-    <row r="93" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A93" s="5"/>
       <c r="B93" s="5" t="s">
         <v>43</v>
@@ -7615,7 +7682,7 @@
       <c r="AL93" s="5"/>
       <c r="AM93" s="5"/>
     </row>
-    <row r="94" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A94" s="5"/>
       <c r="B94" s="5" t="s">
         <v>43</v>
@@ -7682,7 +7749,7 @@
       <c r="AL94" s="5"/>
       <c r="AM94" s="5"/>
     </row>
-    <row r="95" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A95" s="5"/>
       <c r="B95" s="5" t="s">
         <v>43</v>
@@ -7749,7 +7816,7 @@
       <c r="AL95" s="5"/>
       <c r="AM95" s="5"/>
     </row>
-    <row r="96" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A96" s="5"/>
       <c r="B96" s="5" t="s">
         <v>43</v>
@@ -7816,7 +7883,7 @@
       <c r="AL96" s="5"/>
       <c r="AM96" s="5"/>
     </row>
-    <row r="97" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A97" s="5"/>
       <c r="B97" s="5" t="s">
         <v>43</v>
@@ -7885,7 +7952,7 @@
       <c r="AL97" s="5"/>
       <c r="AM97" s="5"/>
     </row>
-    <row r="98" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A98" s="5"/>
       <c r="B98" s="5" t="s">
         <v>43</v>
@@ -7954,7 +8021,7 @@
       <c r="AL98" s="5"/>
       <c r="AM98" s="5"/>
     </row>
-    <row r="99" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A99" s="5"/>
       <c r="B99" s="5" t="s">
         <v>43</v>
@@ -8023,7 +8090,7 @@
       <c r="AL99" s="5"/>
       <c r="AM99" s="5"/>
     </row>
-    <row r="100" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A100" s="5"/>
       <c r="B100" s="5" t="s">
         <v>43</v>
@@ -8092,7 +8159,7 @@
       <c r="AL100" s="5"/>
       <c r="AM100" s="5"/>
     </row>
-    <row r="101" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A101" s="5"/>
       <c r="B101" s="5" t="s">
         <v>43</v>
@@ -8161,7 +8228,7 @@
       <c r="AL101" s="5"/>
       <c r="AM101" s="5"/>
     </row>
-    <row r="102" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A102" s="5"/>
       <c r="B102" s="5" t="s">
         <v>43</v>
@@ -8230,7 +8297,7 @@
       <c r="AL102" s="5"/>
       <c r="AM102" s="5"/>
     </row>
-    <row r="103" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A103" s="5"/>
       <c r="B103" s="5" t="s">
         <v>43</v>
@@ -8299,7 +8366,7 @@
       <c r="AL103" s="5"/>
       <c r="AM103" s="5"/>
     </row>
-    <row r="104" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A104" s="5"/>
       <c r="B104" s="5" t="s">
         <v>43</v>
@@ -8368,7 +8435,7 @@
       <c r="AL104" s="5"/>
       <c r="AM104" s="5"/>
     </row>
-    <row r="105" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A105" s="5"/>
       <c r="B105" s="5" t="s">
         <v>43</v>
@@ -8453,7 +8520,7 @@
       </c>
       <c r="AM105" s="5"/>
     </row>
-    <row r="106" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A106" s="5"/>
       <c r="B106" s="5" t="s">
         <v>43</v>
@@ -8538,7 +8605,7 @@
       </c>
       <c r="AM106" s="5"/>
     </row>
-    <row r="107" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A107" s="5"/>
       <c r="B107" s="5" t="s">
         <v>43</v>
@@ -8623,7 +8690,7 @@
       </c>
       <c r="AM107" s="5"/>
     </row>
-    <row r="108" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A108" s="5"/>
       <c r="B108" s="5" t="s">
         <v>43</v>
@@ -8708,7 +8775,7 @@
       </c>
       <c r="AM108" s="5"/>
     </row>
-    <row r="109" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A109" s="5"/>
       <c r="B109" s="5" t="s">
         <v>43</v>
@@ -8793,7 +8860,7 @@
       </c>
       <c r="AM109" s="5"/>
     </row>
-    <row r="110" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A110" s="5"/>
       <c r="B110" s="5" t="s">
         <v>43</v>
@@ -8878,7 +8945,7 @@
       </c>
       <c r="AM110" s="5"/>
     </row>
-    <row r="111" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A111" s="5"/>
       <c r="B111" s="5" t="s">
         <v>43</v>
@@ -8963,7 +9030,7 @@
       </c>
       <c r="AM111" s="5"/>
     </row>
-    <row r="112" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A112" s="5"/>
       <c r="B112" s="5" t="s">
         <v>43</v>
@@ -9048,7 +9115,7 @@
       </c>
       <c r="AM112" s="5"/>
     </row>
-    <row r="113" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A113" s="5"/>
       <c r="B113" s="5" t="s">
         <v>43</v>
@@ -9133,7 +9200,7 @@
       </c>
       <c r="AM113" s="5"/>
     </row>
-    <row r="114" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A114" s="5"/>
       <c r="B114" s="5" t="s">
         <v>43</v>
@@ -9218,7 +9285,7 @@
       </c>
       <c r="AM114" s="5"/>
     </row>
-    <row r="115" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A115" s="5"/>
       <c r="B115" s="5" t="s">
         <v>43</v>
@@ -9303,7 +9370,7 @@
       </c>
       <c r="AM115" s="5"/>
     </row>
-    <row r="116" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A116" s="5"/>
       <c r="B116" s="5" t="s">
         <v>43</v>
@@ -9388,7 +9455,7 @@
       </c>
       <c r="AM116" s="5"/>
     </row>
-    <row r="117" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A117" s="5"/>
       <c r="B117" s="5" t="s">
         <v>43</v>
@@ -9469,7 +9536,7 @@
       </c>
       <c r="AM117" s="5"/>
     </row>
-    <row r="118" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A118" s="5"/>
       <c r="B118" s="5" t="s">
         <v>43</v>
@@ -9550,7 +9617,7 @@
       </c>
       <c r="AM118" s="5"/>
     </row>
-    <row r="119" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A119" s="5"/>
       <c r="B119" s="5" t="s">
         <v>43</v>
@@ -9631,7 +9698,7 @@
       </c>
       <c r="AM119" s="5"/>
     </row>
-    <row r="120" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A120" s="5"/>
       <c r="B120" s="5" t="s">
         <v>43</v>
@@ -9712,7 +9779,7 @@
       </c>
       <c r="AM120" s="5"/>
     </row>
-    <row r="121" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A121" s="5"/>
       <c r="B121" s="5" t="s">
         <v>43</v>
@@ -9793,7 +9860,7 @@
       </c>
       <c r="AM121" s="5"/>
     </row>
-    <row r="122" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A122" s="5"/>
       <c r="B122" s="5" t="s">
         <v>43</v>
@@ -9874,7 +9941,7 @@
       </c>
       <c r="AM122" s="5"/>
     </row>
-    <row r="123" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A123" s="5"/>
       <c r="B123" s="5" t="s">
         <v>43</v>
@@ -9955,7 +10022,7 @@
       </c>
       <c r="AM123" s="5"/>
     </row>
-    <row r="124" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A124" s="5"/>
       <c r="B124" s="5" t="s">
         <v>43</v>
@@ -10036,7 +10103,7 @@
       </c>
       <c r="AM124" s="5"/>
     </row>
-    <row r="125" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A125" s="5"/>
       <c r="B125" s="5" t="s">
         <v>43</v>
@@ -10115,7 +10182,7 @@
       </c>
       <c r="AM125" s="5"/>
     </row>
-    <row r="126" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A126" s="5"/>
       <c r="B126" s="5" t="s">
         <v>43</v>
@@ -10196,7 +10263,7 @@
       </c>
       <c r="AM126" s="5"/>
     </row>
-    <row r="127" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A127" s="5"/>
       <c r="B127" s="5" t="s">
         <v>43</v>
@@ -10277,7 +10344,7 @@
       </c>
       <c r="AM127" s="5"/>
     </row>
-    <row r="128" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A128" s="5"/>
       <c r="B128" s="5" t="s">
         <v>43</v>
@@ -10358,7 +10425,7 @@
       </c>
       <c r="AM128" s="5"/>
     </row>
-    <row r="129" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A129" s="5"/>
       <c r="B129" s="5" t="s">
         <v>43</v>
@@ -10429,7 +10496,7 @@
       <c r="AL129" s="5"/>
       <c r="AM129" s="5"/>
     </row>
-    <row r="130" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A130" s="5"/>
       <c r="B130" s="5" t="s">
         <v>43</v>
@@ -10500,7 +10567,7 @@
       <c r="AL130" s="5"/>
       <c r="AM130" s="5"/>
     </row>
-    <row r="131" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A131" s="5"/>
       <c r="B131" s="5" t="s">
         <v>43</v>
@@ -10571,7 +10638,7 @@
       <c r="AL131" s="5"/>
       <c r="AM131" s="5"/>
     </row>
-    <row r="132" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A132" s="5"/>
       <c r="B132" s="5" t="s">
         <v>43</v>
@@ -10642,7 +10709,7 @@
       <c r="AL132" s="5"/>
       <c r="AM132" s="5"/>
     </row>
-    <row r="133" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A133" s="5"/>
       <c r="B133" s="5" t="s">
         <v>43</v>
@@ -10713,7 +10780,7 @@
       <c r="AL133" s="5"/>
       <c r="AM133" s="5"/>
     </row>
-    <row r="134" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A134" s="5"/>
       <c r="B134" s="5" t="s">
         <v>43</v>
@@ -10784,7 +10851,7 @@
       <c r="AL134" s="5"/>
       <c r="AM134" s="5"/>
     </row>
-    <row r="135" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A135" s="5"/>
       <c r="B135" s="5" t="s">
         <v>43</v>
@@ -10855,7 +10922,7 @@
       <c r="AL135" s="5"/>
       <c r="AM135" s="5"/>
     </row>
-    <row r="136" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A136" s="5"/>
       <c r="B136" s="5" t="s">
         <v>43</v>
@@ -10926,7 +10993,7 @@
       <c r="AL136" s="5"/>
       <c r="AM136" s="5"/>
     </row>
-    <row r="137" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A137" s="5"/>
       <c r="B137" s="5" t="s">
         <v>43</v>
@@ -10997,7 +11064,7 @@
       <c r="AL137" s="5"/>
       <c r="AM137" s="5"/>
     </row>
-    <row r="138" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A138" s="5"/>
       <c r="B138" s="5" t="s">
         <v>43</v>
@@ -11068,7 +11135,7 @@
       <c r="AL138" s="5"/>
       <c r="AM138" s="5"/>
     </row>
-    <row r="139" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A139" s="5"/>
       <c r="B139" s="5" t="s">
         <v>43</v>
@@ -11139,7 +11206,7 @@
       <c r="AL139" s="5"/>
       <c r="AM139" s="5"/>
     </row>
-    <row r="140" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A140" s="5"/>
       <c r="B140" s="5" t="s">
         <v>43</v>
@@ -11210,7 +11277,7 @@
       <c r="AL140" s="5"/>
       <c r="AM140" s="5"/>
     </row>
-    <row r="141" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A141" s="5"/>
       <c r="B141" s="5" t="s">
         <v>43</v>
@@ -11291,7 +11358,7 @@
       </c>
       <c r="AM141" s="5"/>
     </row>
-    <row r="142" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A142" s="5"/>
       <c r="B142" s="5" t="s">
         <v>43</v>
@@ -11372,7 +11439,7 @@
       </c>
       <c r="AM142" s="5"/>
     </row>
-    <row r="143" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A143" s="5"/>
       <c r="B143" s="5" t="s">
         <v>43</v>
@@ -11453,7 +11520,7 @@
       </c>
       <c r="AM143" s="5"/>
     </row>
-    <row r="144" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A144" s="5"/>
       <c r="B144" s="5" t="s">
         <v>43</v>
@@ -11534,7 +11601,7 @@
       </c>
       <c r="AM144" s="5"/>
     </row>
-    <row r="145" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A145" s="5"/>
       <c r="B145" s="5" t="s">
         <v>43</v>
@@ -11615,7 +11682,7 @@
       </c>
       <c r="AM145" s="5"/>
     </row>
-    <row r="146" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A146" s="5"/>
       <c r="B146" s="5" t="s">
         <v>43</v>
@@ -11696,7 +11763,7 @@
       </c>
       <c r="AM146" s="5"/>
     </row>
-    <row r="147" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A147" s="5"/>
       <c r="B147" s="5" t="s">
         <v>43</v>
@@ -11777,7 +11844,7 @@
       </c>
       <c r="AM147" s="5"/>
     </row>
-    <row r="148" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A148" s="5"/>
       <c r="B148" s="5" t="s">
         <v>43</v>
@@ -11858,7 +11925,7 @@
       </c>
       <c r="AM148" s="5"/>
     </row>
-    <row r="149" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A149" s="5"/>
       <c r="B149" s="5" t="s">
         <v>43</v>
@@ -11939,7 +12006,7 @@
       </c>
       <c r="AM149" s="5"/>
     </row>
-    <row r="150" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A150" s="5"/>
       <c r="B150" s="5" t="s">
         <v>43</v>
@@ -12020,7 +12087,7 @@
       </c>
       <c r="AM150" s="5"/>
     </row>
-    <row r="151" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A151" s="5"/>
       <c r="B151" s="5" t="s">
         <v>43</v>
@@ -12101,7 +12168,7 @@
       </c>
       <c r="AM151" s="5"/>
     </row>
-    <row r="152" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A152" s="5"/>
       <c r="B152" s="5" t="s">
         <v>43</v>
@@ -12182,7 +12249,7 @@
       </c>
       <c r="AM152" s="5"/>
     </row>
-    <row r="153" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A153" s="5"/>
       <c r="B153" s="5" t="s">
         <v>43</v>
@@ -12251,7 +12318,7 @@
       <c r="AL153" s="5"/>
       <c r="AM153" s="5"/>
     </row>
-    <row r="154" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A154" s="5"/>
       <c r="B154" s="5" t="s">
         <v>43</v>
@@ -12320,7 +12387,7 @@
       <c r="AL154" s="5"/>
       <c r="AM154" s="5"/>
     </row>
-    <row r="155" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A155" s="5"/>
       <c r="B155" s="5" t="s">
         <v>43</v>
@@ -12389,7 +12456,7 @@
       <c r="AL155" s="5"/>
       <c r="AM155" s="5"/>
     </row>
-    <row r="156" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A156" s="5"/>
       <c r="B156" s="5" t="s">
         <v>43</v>
@@ -12458,7 +12525,7 @@
       <c r="AL156" s="5"/>
       <c r="AM156" s="5"/>
     </row>
-    <row r="157" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A157" s="5"/>
       <c r="B157" s="5" t="s">
         <v>43</v>
@@ -12527,7 +12594,7 @@
       <c r="AL157" s="5"/>
       <c r="AM157" s="5"/>
     </row>
-    <row r="158" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A158" s="5"/>
       <c r="B158" s="5" t="s">
         <v>43</v>
@@ -12596,7 +12663,7 @@
       <c r="AL158" s="5"/>
       <c r="AM158" s="5"/>
     </row>
-    <row r="159" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A159" s="5"/>
       <c r="B159" s="5" t="s">
         <v>43</v>
@@ -12665,7 +12732,7 @@
       <c r="AL159" s="5"/>
       <c r="AM159" s="5"/>
     </row>
-    <row r="160" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A160" s="5"/>
       <c r="B160" s="5" t="s">
         <v>43</v>
@@ -12736,7 +12803,7 @@
       <c r="AL160" s="5"/>
       <c r="AM160" s="5"/>
     </row>
-    <row r="161" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A161" s="5"/>
       <c r="B161" s="5" t="s">
         <v>43</v>
@@ -12807,7 +12874,7 @@
       <c r="AL161" s="5"/>
       <c r="AM161" s="5"/>
     </row>
-    <row r="162" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A162" s="5"/>
       <c r="B162" s="5" t="s">
         <v>43</v>
@@ -12878,7 +12945,7 @@
       <c r="AL162" s="5"/>
       <c r="AM162" s="5"/>
     </row>
-    <row r="163" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A163" s="5"/>
       <c r="B163" s="5" t="s">
         <v>43</v>
@@ -12949,7 +13016,7 @@
       <c r="AL163" s="5"/>
       <c r="AM163" s="5"/>
     </row>
-    <row r="164" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A164" s="5"/>
       <c r="B164" s="5" t="s">
         <v>43</v>
@@ -13020,7 +13087,7 @@
       <c r="AL164" s="5"/>
       <c r="AM164" s="5"/>
     </row>
-    <row r="165" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A165" s="5"/>
       <c r="B165" s="5" t="s">
         <v>43</v>
@@ -13091,7 +13158,7 @@
       <c r="AL165" s="5"/>
       <c r="AM165" s="5"/>
     </row>
-    <row r="166" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A166" s="5"/>
       <c r="B166" s="5" t="s">
         <v>43</v>
@@ -13162,7 +13229,7 @@
       <c r="AL166" s="5"/>
       <c r="AM166" s="5"/>
     </row>
-    <row r="167" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A167" s="5"/>
       <c r="B167" s="5" t="s">
         <v>43</v>
@@ -13233,7 +13300,7 @@
       <c r="AL167" s="5"/>
       <c r="AM167" s="5"/>
     </row>
-    <row r="168" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A168" s="5"/>
       <c r="B168" s="5" t="s">
         <v>43</v>
@@ -13304,7 +13371,7 @@
       <c r="AL168" s="5"/>
       <c r="AM168" s="5"/>
     </row>
-    <row r="169" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A169" s="5"/>
       <c r="B169" s="5" t="s">
         <v>43</v>
@@ -13375,7 +13442,7 @@
       <c r="AL169" s="5"/>
       <c r="AM169" s="5"/>
     </row>
-    <row r="170" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A170" s="5"/>
       <c r="B170" s="5" t="s">
         <v>43</v>
@@ -13446,7 +13513,7 @@
       <c r="AL170" s="5"/>
       <c r="AM170" s="5"/>
     </row>
-    <row r="171" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A171" s="5"/>
       <c r="B171" s="5" t="s">
         <v>43</v>
@@ -13517,7 +13584,7 @@
       <c r="AL171" s="5"/>
       <c r="AM171" s="5"/>
     </row>
-    <row r="172" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A172" s="5"/>
       <c r="B172" s="5" t="s">
         <v>43</v>
@@ -13602,7 +13669,7 @@
       </c>
       <c r="AM172" s="5"/>
     </row>
-    <row r="173" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A173" s="5"/>
       <c r="B173" s="5" t="s">
         <v>43</v>
@@ -13687,7 +13754,7 @@
       </c>
       <c r="AM173" s="5"/>
     </row>
-    <row r="174" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A174" s="5"/>
       <c r="B174" s="5" t="s">
         <v>43</v>
@@ -13772,7 +13839,7 @@
       </c>
       <c r="AM174" s="5"/>
     </row>
-    <row r="175" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A175" s="5"/>
       <c r="B175" s="5" t="s">
         <v>43</v>
@@ -13857,7 +13924,7 @@
       </c>
       <c r="AM175" s="5"/>
     </row>
-    <row r="176" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A176" s="5"/>
       <c r="B176" s="5" t="s">
         <v>43</v>
@@ -13942,7 +14009,7 @@
       </c>
       <c r="AM176" s="5"/>
     </row>
-    <row r="177" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A177" s="5"/>
       <c r="B177" s="5" t="s">
         <v>43</v>
@@ -14027,7 +14094,7 @@
       </c>
       <c r="AM177" s="5"/>
     </row>
-    <row r="178" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A178" s="5"/>
       <c r="B178" s="5" t="s">
         <v>43</v>
@@ -14112,7 +14179,7 @@
       </c>
       <c r="AM178" s="5"/>
     </row>
-    <row r="179" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A179" s="5"/>
       <c r="B179" s="5" t="s">
         <v>43</v>
@@ -14197,7 +14264,7 @@
       </c>
       <c r="AM179" s="5"/>
     </row>
-    <row r="180" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A180" s="5"/>
       <c r="B180" s="5" t="s">
         <v>43</v>
@@ -14282,7 +14349,7 @@
       </c>
       <c r="AM180" s="5"/>
     </row>
-    <row r="181" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A181" s="5"/>
       <c r="B181" s="5" t="s">
         <v>43</v>
@@ -14367,7 +14434,7 @@
       </c>
       <c r="AM181" s="5"/>
     </row>
-    <row r="182" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A182" s="5"/>
       <c r="B182" s="5" t="s">
         <v>43</v>
@@ -14452,7 +14519,7 @@
       </c>
       <c r="AM182" s="5"/>
     </row>
-    <row r="183" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A183" s="5"/>
       <c r="B183" s="5" t="s">
         <v>43</v>
@@ -14537,7 +14604,7 @@
       </c>
       <c r="AM183" s="5"/>
     </row>
-    <row r="184" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A184" s="5"/>
       <c r="B184" s="5" t="s">
         <v>43</v>
@@ -14606,7 +14673,7 @@
       <c r="AL184" s="5"/>
       <c r="AM184" s="5"/>
     </row>
-    <row r="185" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A185" s="5"/>
       <c r="B185" s="5" t="s">
         <v>43</v>
@@ -14675,7 +14742,7 @@
       <c r="AL185" s="5"/>
       <c r="AM185" s="5"/>
     </row>
-    <row r="186" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A186" s="5"/>
       <c r="B186" s="5" t="s">
         <v>43</v>
@@ -14744,7 +14811,7 @@
       <c r="AL186" s="5"/>
       <c r="AM186" s="5"/>
     </row>
-    <row r="187" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A187" s="5"/>
       <c r="B187" s="5" t="s">
         <v>43</v>
@@ -14813,7 +14880,7 @@
       <c r="AL187" s="5"/>
       <c r="AM187" s="5"/>
     </row>
-    <row r="188" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A188" s="5"/>
       <c r="B188" s="5" t="s">
         <v>43</v>
@@ -14882,7 +14949,7 @@
       <c r="AL188" s="5"/>
       <c r="AM188" s="5"/>
     </row>
-    <row r="189" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A189" s="5"/>
       <c r="B189" s="5" t="s">
         <v>43</v>
@@ -14951,7 +15018,7 @@
       <c r="AL189" s="5"/>
       <c r="AM189" s="5"/>
     </row>
-    <row r="190" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A190" s="5"/>
       <c r="B190" s="5" t="s">
         <v>43</v>
@@ -15020,7 +15087,7 @@
       <c r="AL190" s="5"/>
       <c r="AM190" s="5"/>
     </row>
-    <row r="191" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A191" s="5"/>
       <c r="B191" s="5" t="s">
         <v>43</v>
@@ -15091,7 +15158,7 @@
       <c r="AL191" s="5"/>
       <c r="AM191" s="5"/>
     </row>
-    <row r="192" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A192" s="5"/>
       <c r="B192" s="5" t="s">
         <v>43</v>
@@ -15162,7 +15229,7 @@
       <c r="AL192" s="5"/>
       <c r="AM192" s="5"/>
     </row>
-    <row r="193" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A193" s="5"/>
       <c r="B193" s="5" t="s">
         <v>43</v>
@@ -15233,7 +15300,7 @@
       <c r="AL193" s="5"/>
       <c r="AM193" s="5"/>
     </row>
-    <row r="194" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A194" s="5"/>
       <c r="B194" s="5" t="s">
         <v>43</v>
@@ -15304,7 +15371,7 @@
       <c r="AL194" s="5"/>
       <c r="AM194" s="5"/>
     </row>
-    <row r="195" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A195" s="5"/>
       <c r="B195" s="5" t="s">
         <v>43</v>
@@ -15375,7 +15442,7 @@
       <c r="AL195" s="5"/>
       <c r="AM195" s="5"/>
     </row>
-    <row r="196" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A196" s="5"/>
       <c r="B196" s="5" t="s">
         <v>43</v>
@@ -15446,7 +15513,7 @@
       <c r="AL196" s="5"/>
       <c r="AM196" s="5"/>
     </row>
-    <row r="197" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A197" s="5"/>
       <c r="B197" s="5" t="s">
         <v>43</v>
@@ -15517,7 +15584,7 @@
       <c r="AL197" s="5"/>
       <c r="AM197" s="5"/>
     </row>
-    <row r="198" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A198" s="5"/>
       <c r="B198" s="5" t="s">
         <v>43</v>
@@ -15588,7 +15655,7 @@
       <c r="AL198" s="5"/>
       <c r="AM198" s="5"/>
     </row>
-    <row r="199" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A199" s="5"/>
       <c r="B199" s="5" t="s">
         <v>43</v>
@@ -15659,7 +15726,7 @@
       <c r="AL199" s="5"/>
       <c r="AM199" s="5"/>
     </row>
-    <row r="200" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A200" s="5"/>
       <c r="B200" s="5" t="s">
         <v>43</v>
@@ -15730,7 +15797,7 @@
       <c r="AL200" s="5"/>
       <c r="AM200" s="5"/>
     </row>
-    <row r="201" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A201" s="5"/>
       <c r="B201" s="5" t="s">
         <v>43</v>
@@ -15801,7 +15868,7 @@
       <c r="AL201" s="5"/>
       <c r="AM201" s="5"/>
     </row>
-    <row r="202" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A202" s="5"/>
       <c r="B202" s="5" t="s">
         <v>43</v>
@@ -15872,7 +15939,7 @@
       <c r="AL202" s="5"/>
       <c r="AM202" s="5"/>
     </row>
-    <row r="203" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A203" s="5"/>
       <c r="B203" s="5" t="s">
         <v>43</v>
@@ -15941,7 +16008,7 @@
       <c r="AL203" s="5"/>
       <c r="AM203" s="5"/>
     </row>
-    <row r="204" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A204" s="5"/>
       <c r="B204" s="5" t="s">
         <v>43</v>
@@ -16010,7 +16077,7 @@
       <c r="AL204" s="5"/>
       <c r="AM204" s="5"/>
     </row>
-    <row r="205" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A205" s="5"/>
       <c r="B205" s="5" t="s">
         <v>43</v>
@@ -16079,7 +16146,7 @@
       <c r="AL205" s="5"/>
       <c r="AM205" s="5"/>
     </row>
-    <row r="206" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A206" s="5"/>
       <c r="B206" s="5" t="s">
         <v>43</v>
@@ -16148,7 +16215,7 @@
       <c r="AL206" s="5"/>
       <c r="AM206" s="5"/>
     </row>
-    <row r="207" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A207" s="5"/>
       <c r="B207" s="5" t="s">
         <v>43</v>
@@ -16217,7 +16284,7 @@
       <c r="AL207" s="5"/>
       <c r="AM207" s="5"/>
     </row>
-    <row r="208" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A208" s="5"/>
       <c r="B208" s="5" t="s">
         <v>43</v>
@@ -16286,7 +16353,7 @@
       <c r="AL208" s="5"/>
       <c r="AM208" s="5"/>
     </row>
-    <row r="209" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A209" s="5"/>
       <c r="B209" s="5" t="s">
         <v>43</v>
@@ -16355,7 +16422,7 @@
       <c r="AL209" s="5"/>
       <c r="AM209" s="5"/>
     </row>
-    <row r="210" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A210" s="5"/>
       <c r="B210" s="5" t="s">
         <v>43</v>
@@ -16436,7 +16503,7 @@
       </c>
       <c r="AM210" s="5"/>
     </row>
-    <row r="211" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A211" s="5"/>
       <c r="B211" s="5" t="s">
         <v>43</v>
@@ -16517,7 +16584,7 @@
       </c>
       <c r="AM211" s="5"/>
     </row>
-    <row r="212" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A212" s="5"/>
       <c r="B212" s="5" t="s">
         <v>43</v>
@@ -16598,7 +16665,7 @@
       </c>
       <c r="AM212" s="5"/>
     </row>
-    <row r="213" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A213" s="5"/>
       <c r="B213" s="5" t="s">
         <v>43</v>
@@ -16679,7 +16746,7 @@
       </c>
       <c r="AM213" s="5"/>
     </row>
-    <row r="214" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A214" s="5"/>
       <c r="B214" s="5" t="s">
         <v>43</v>
@@ -16760,7 +16827,7 @@
       </c>
       <c r="AM214" s="5"/>
     </row>
-    <row r="215" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A215" s="5"/>
       <c r="B215" s="5" t="s">
         <v>43</v>
@@ -16841,7 +16908,7 @@
       </c>
       <c r="AM215" s="5"/>
     </row>
-    <row r="216" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A216" s="5"/>
       <c r="B216" s="5" t="s">
         <v>43</v>
@@ -16922,7 +16989,7 @@
       </c>
       <c r="AM216" s="5"/>
     </row>
-    <row r="217" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A217" s="5"/>
       <c r="B217" s="5" t="s">
         <v>43</v>
@@ -17003,7 +17070,7 @@
       </c>
       <c r="AM217" s="5"/>
     </row>
-    <row r="218" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A218" s="5"/>
       <c r="B218" s="5" t="s">
         <v>43</v>
@@ -17084,7 +17151,7 @@
       </c>
       <c r="AM218" s="5"/>
     </row>
-    <row r="219" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A219" s="5"/>
       <c r="B219" s="5" t="s">
         <v>43</v>
@@ -17165,7 +17232,7 @@
       </c>
       <c r="AM219" s="5"/>
     </row>
-    <row r="220" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A220" s="5"/>
       <c r="B220" s="5" t="s">
         <v>43</v>
@@ -17246,7 +17313,7 @@
       </c>
       <c r="AM220" s="5"/>
     </row>
-    <row r="221" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A221" s="5"/>
       <c r="B221" s="5" t="s">
         <v>43</v>
@@ -17327,7 +17394,7 @@
       </c>
       <c r="AM221" s="5"/>
     </row>
-    <row r="222" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A222" s="5"/>
       <c r="B222" s="5" t="s">
         <v>43</v>
@@ -17396,7 +17463,7 @@
       <c r="AL222" s="5"/>
       <c r="AM222" s="5"/>
     </row>
-    <row r="223" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A223" s="5"/>
       <c r="B223" s="5" t="s">
         <v>43</v>
@@ -17465,7 +17532,7 @@
       <c r="AL223" s="5"/>
       <c r="AM223" s="5"/>
     </row>
-    <row r="224" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A224" s="5"/>
       <c r="B224" s="5" t="s">
         <v>43</v>
@@ -17534,7 +17601,7 @@
       <c r="AL224" s="5"/>
       <c r="AM224" s="5"/>
     </row>
-    <row r="225" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A225" s="5"/>
       <c r="B225" s="5" t="s">
         <v>43</v>
@@ -17603,7 +17670,7 @@
       <c r="AL225" s="5"/>
       <c r="AM225" s="5"/>
     </row>
-    <row r="226" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A226" s="5"/>
       <c r="B226" s="5" t="s">
         <v>43</v>
@@ -17672,7 +17739,7 @@
       <c r="AL226" s="5"/>
       <c r="AM226" s="5"/>
     </row>
-    <row r="227" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A227" s="5"/>
       <c r="B227" s="5" t="s">
         <v>43</v>
@@ -17741,7 +17808,7 @@
       <c r="AL227" s="5"/>
       <c r="AM227" s="5"/>
     </row>
-    <row r="228" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A228" s="5"/>
       <c r="B228" s="5" t="s">
         <v>43</v>
@@ -17810,7 +17877,7 @@
       <c r="AL228" s="5"/>
       <c r="AM228" s="5"/>
     </row>
-    <row r="229" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A229" s="5"/>
       <c r="B229" s="5" t="s">
         <v>43</v>
@@ -17885,7 +17952,7 @@
       <c r="AL229" s="5"/>
       <c r="AM229" s="5"/>
     </row>
-    <row r="230" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A230" s="5"/>
       <c r="B230" s="5" t="s">
         <v>43</v>
@@ -17960,7 +18027,7 @@
       <c r="AL230" s="5"/>
       <c r="AM230" s="5"/>
     </row>
-    <row r="231" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A231" s="5"/>
       <c r="B231" s="5" t="s">
         <v>43</v>
@@ -18035,7 +18102,7 @@
       <c r="AL231" s="5"/>
       <c r="AM231" s="5"/>
     </row>
-    <row r="232" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A232" s="5"/>
       <c r="B232" s="5" t="s">
         <v>43</v>
@@ -18110,7 +18177,7 @@
       <c r="AL232" s="5"/>
       <c r="AM232" s="5"/>
     </row>
-    <row r="233" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A233" s="5"/>
       <c r="B233" s="5" t="s">
         <v>43</v>
@@ -18185,7 +18252,7 @@
       <c r="AL233" s="5"/>
       <c r="AM233" s="5"/>
     </row>
-    <row r="234" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A234" s="5"/>
       <c r="B234" s="5" t="s">
         <v>43</v>
@@ -18260,7 +18327,7 @@
       <c r="AL234" s="5"/>
       <c r="AM234" s="5"/>
     </row>
-    <row r="235" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A235" s="5"/>
       <c r="B235" s="5" t="s">
         <v>43</v>
@@ -18331,7 +18398,7 @@
       <c r="AL235" s="5"/>
       <c r="AM235" s="5"/>
     </row>
-    <row r="236" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="236" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A236" s="5"/>
       <c r="B236" s="5" t="s">
         <v>43</v>
@@ -18402,7 +18469,7 @@
       <c r="AL236" s="5"/>
       <c r="AM236" s="5"/>
     </row>
-    <row r="237" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="237" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A237" s="5"/>
       <c r="B237" s="5" t="s">
         <v>43</v>
@@ -18473,7 +18540,7 @@
       <c r="AL237" s="5"/>
       <c r="AM237" s="5"/>
     </row>
-    <row r="238" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="238" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A238" s="5"/>
       <c r="B238" s="5" t="s">
         <v>43</v>
@@ -18544,7 +18611,7 @@
       <c r="AL238" s="5"/>
       <c r="AM238" s="5"/>
     </row>
-    <row r="239" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="239" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A239" s="5"/>
       <c r="B239" s="5" t="s">
         <v>43</v>
@@ -18615,7 +18682,7 @@
       <c r="AL239" s="5"/>
       <c r="AM239" s="5"/>
     </row>
-    <row r="240" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="240" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A240" s="5"/>
       <c r="B240" s="5" t="s">
         <v>43</v>
@@ -18686,7 +18753,7 @@
       <c r="AL240" s="5"/>
       <c r="AM240" s="5"/>
     </row>
-    <row r="241" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="241" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A241" s="5"/>
       <c r="B241" s="5" t="s">
         <v>43</v>
@@ -18767,7 +18834,7 @@
       </c>
       <c r="AM241" s="5"/>
     </row>
-    <row r="242" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="242" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A242" s="5"/>
       <c r="B242" s="5" t="s">
         <v>43</v>
@@ -18848,7 +18915,7 @@
       </c>
       <c r="AM242" s="5"/>
     </row>
-    <row r="243" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A243" s="5"/>
       <c r="B243" s="5" t="s">
         <v>43</v>
@@ -18929,7 +18996,7 @@
       </c>
       <c r="AM243" s="5"/>
     </row>
-    <row r="244" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="244" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A244" s="5"/>
       <c r="B244" s="5" t="s">
         <v>43</v>
@@ -19010,7 +19077,7 @@
       </c>
       <c r="AM244" s="5"/>
     </row>
-    <row r="245" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="245" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A245" s="5"/>
       <c r="B245" s="5" t="s">
         <v>43</v>
@@ -19091,7 +19158,7 @@
       </c>
       <c r="AM245" s="5"/>
     </row>
-    <row r="246" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A246" s="5"/>
       <c r="B246" s="5" t="s">
         <v>43</v>
@@ -19172,7 +19239,7 @@
       </c>
       <c r="AM246" s="5"/>
     </row>
-    <row r="247" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="247" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A247" s="5"/>
       <c r="B247" s="5" t="s">
         <v>43</v>
@@ -19239,7 +19306,7 @@
       <c r="AL247" s="5"/>
       <c r="AM247" s="5"/>
     </row>
-    <row r="248" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="248" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A248" s="5"/>
       <c r="B248" s="5" t="s">
         <v>43</v>
@@ -19306,7 +19373,7 @@
       <c r="AL248" s="5"/>
       <c r="AM248" s="5"/>
     </row>
-    <row r="249" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="249" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A249" s="5"/>
       <c r="B249" s="5" t="s">
         <v>43</v>
@@ -19373,7 +19440,7 @@
       <c r="AL249" s="5"/>
       <c r="AM249" s="5"/>
     </row>
-    <row r="250" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="250" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A250" s="5"/>
       <c r="B250" s="5" t="s">
         <v>43</v>
@@ -19440,7 +19507,7 @@
       <c r="AL250" s="5"/>
       <c r="AM250" s="5"/>
     </row>
-    <row r="251" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="251" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A251" s="5"/>
       <c r="B251" s="5" t="s">
         <v>43</v>
@@ -19507,7 +19574,7 @@
       <c r="AL251" s="5"/>
       <c r="AM251" s="5"/>
     </row>
-    <row r="252" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="252" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A252" s="5"/>
       <c r="B252" s="5" t="s">
         <v>43</v>
@@ -19574,7 +19641,7 @@
       <c r="AL252" s="5"/>
       <c r="AM252" s="5"/>
     </row>
-    <row r="253" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="253" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A253" s="5"/>
       <c r="B253" s="5" t="s">
         <v>43</v>
@@ -19641,7 +19708,7 @@
       <c r="AL253" s="5"/>
       <c r="AM253" s="5"/>
     </row>
-    <row r="254" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="254" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A254" s="5"/>
       <c r="B254" s="5" t="s">
         <v>43</v>
@@ -19710,7 +19777,7 @@
       <c r="AL254" s="5"/>
       <c r="AM254" s="5"/>
     </row>
-    <row r="255" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="255" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A255" s="5"/>
       <c r="B255" s="5" t="s">
         <v>43</v>
@@ -19779,7 +19846,7 @@
       <c r="AL255" s="5"/>
       <c r="AM255" s="5"/>
     </row>
-    <row r="256" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="256" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A256" s="5"/>
       <c r="B256" s="5" t="s">
         <v>43</v>
@@ -19848,7 +19915,7 @@
       <c r="AL256" s="5"/>
       <c r="AM256" s="5"/>
     </row>
-    <row r="257" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="257" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A257" s="5"/>
       <c r="B257" s="5" t="s">
         <v>43</v>
@@ -19917,7 +19984,7 @@
       <c r="AL257" s="5"/>
       <c r="AM257" s="5"/>
     </row>
-    <row r="258" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="258" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A258" s="5"/>
       <c r="B258" s="5" t="s">
         <v>43</v>
@@ -19986,7 +20053,7 @@
       <c r="AL258" s="5"/>
       <c r="AM258" s="5"/>
     </row>
-    <row r="259" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="259" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A259" s="5"/>
       <c r="B259" s="5" t="s">
         <v>43</v>
@@ -20055,7 +20122,7 @@
       <c r="AL259" s="5"/>
       <c r="AM259" s="5"/>
     </row>
-    <row r="260" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="260" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A260" s="5"/>
       <c r="B260" s="5" t="s">
         <v>43</v>
@@ -20124,7 +20191,7 @@
       <c r="AL260" s="5"/>
       <c r="AM260" s="5"/>
     </row>
-    <row r="261" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="261" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A261" s="5"/>
       <c r="B261" s="5" t="s">
         <v>43</v>
@@ -20205,7 +20272,7 @@
       </c>
       <c r="AM261" s="5"/>
     </row>
-    <row r="262" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="262" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A262" s="5"/>
       <c r="B262" s="5" t="s">
         <v>43</v>
@@ -20286,7 +20353,7 @@
       </c>
       <c r="AM262" s="5"/>
     </row>
-    <row r="263" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="263" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A263" s="5"/>
       <c r="B263" s="5" t="s">
         <v>43</v>
@@ -20367,7 +20434,7 @@
       </c>
       <c r="AM263" s="5"/>
     </row>
-    <row r="264" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="264" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A264" s="5"/>
       <c r="B264" s="5" t="s">
         <v>43</v>
@@ -20448,7 +20515,7 @@
       </c>
       <c r="AM264" s="5"/>
     </row>
-    <row r="265" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="265" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A265" s="5"/>
       <c r="B265" s="5" t="s">
         <v>43</v>
@@ -20529,7 +20596,7 @@
       </c>
       <c r="AM265" s="5"/>
     </row>
-    <row r="266" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="266" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A266" s="5"/>
       <c r="B266" s="5" t="s">
         <v>43</v>
@@ -20610,7 +20677,7 @@
       </c>
       <c r="AM266" s="5"/>
     </row>
-    <row r="267" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="267" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A267" s="5"/>
       <c r="B267" s="5" t="s">
         <v>43</v>
@@ -20691,7 +20758,7 @@
       </c>
       <c r="AM267" s="5"/>
     </row>
-    <row r="268" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="268" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A268" s="5"/>
       <c r="B268" s="5" t="s">
         <v>43</v>
@@ -20772,7 +20839,7 @@
       </c>
       <c r="AM268" s="5"/>
     </row>
-    <row r="269" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="269" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A269" s="5"/>
       <c r="B269" s="5" t="s">
         <v>43</v>
@@ -20853,7 +20920,7 @@
       </c>
       <c r="AM269" s="5"/>
     </row>
-    <row r="270" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="270" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A270" s="5"/>
       <c r="B270" s="5" t="s">
         <v>43</v>
@@ -20934,7 +21001,7 @@
       </c>
       <c r="AM270" s="5"/>
     </row>
-    <row r="271" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="271" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A271" s="5"/>
       <c r="B271" s="5" t="s">
         <v>43</v>
@@ -21015,7 +21082,7 @@
       </c>
       <c r="AM271" s="5"/>
     </row>
-    <row r="272" spans="1:39" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="272" spans="1:39" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A272" s="5"/>
       <c r="B272" s="5" t="s">
         <v>43</v>
@@ -21097,6 +21164,8 @@
       <c r="AM272" s="5"/>
     </row>
   </sheetData>
+  <autoFilter ref="A1:AQ272" xr:uid="{C3395A04-AF43-4335-9FBC-13D8E09A4DF0}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>